<commit_message>
Updated EOL Recovery parameter
</commit_message>
<xml_diff>
--- a/docs/Files/ODYM_Tutorial6_EoLRecoveryRateLL_V1.0.xlsx
+++ b/docs/Files/ODYM_Tutorial6_EoLRecoveryRateLL_V1.0.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28827"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56A8F294-4C16-4DA4-A487-0A98D50ADE5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C769219-D9A5-4CF0-BDE8-DACBEAE8E2A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1222,7 +1222,7 @@
         <v>108</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="F2">
         <v>1</v>
@@ -1251,7 +1251,7 @@
         <v>109</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="F3">
         <v>1</v>

</xml_diff>